<commit_message>
Clase de 29 de Agosto, taller de pregunta tipo examen y presentación del taller final.
</commit_message>
<xml_diff>
--- a/practicaPOO/tallerFinal/Ejercicio2/inventario.xlsx
+++ b/practicaPOO/tallerFinal/Ejercicio2/inventario.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,71 @@
         <v>200</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Maruchan</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nestea</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fuse-tea</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>La lechera-Entera</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Don Vitorio</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>